<commit_message>
Fix màn Quản lý Đèn biển + [F-155] Biểu 08-N: Thống kê hệ thống đèn biển
</commit_message>
<xml_diff>
--- a/src/main/resources/public/template_export/BCKCHT_170.xlsx
+++ b/src/main/resources/public/template_export/BCKCHT_170.xlsx
@@ -235,15 +235,6 @@
     <t>${item.dienTichSuDungTram.asText()}</t>
   </si>
   <si>
-    <t>${thiz.getCateOtherText('AUTH_ORG',item.donViQuanLy.asText())}</t>
-  </si>
-  <si>
-    <t>${thiz.getCateOtherText('DM_APP_PARAM',item.chungLoaiDenChinh.asText(), 'CHUNG_LOAI_DEN')}</t>
-  </si>
-  <si>
-    <t>${thiz.getCateOtherText('DM_APP_PARAM',item.chungLoaiDenDuPhong.asText(), 'CHUNG_LOAI_DEN')}</t>
-  </si>
-  <si>
     <t>Cục Hàng hải và Đường thủy Việt Nam (Phòng KCHT)</t>
   </si>
   <si>
@@ -269,6 +260,15 @@
   </si>
   <si>
     <t>${item.ten.asText()}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('DM_APP_PARAM',item.chungLoaiDenChinh.asText(), 'CHUNG_LOAI_DEN')}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('DM_APP_PARAM',item.chungLoaiDenDuPhong.asText(), 'CHUNG_LOAI_DEN')}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('AUTH_ORG',item.donViQuanLy.asText())}</t>
   </si>
 </sst>
 </file>
@@ -423,32 +423,32 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -729,12 +729,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R18"/>
-  <sheetFormatPr defaultRowHeight="12.75" ns2:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="26.140625" style="1" customWidth="1"/>
@@ -742,111 +742,111 @@
     <col min="19" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
       <c r="D1" s="13"/>
       <c r="E1" s="13"/>
-      <c r="M1" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-    </row>
-    <row r="2" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="M1" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
-      <c r="M2" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-    </row>
-    <row r="3" spans="1:18" ht="12.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
+      <c r="M2" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+    </row>
+    <row r="3" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
-      <c r="M3" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28"/>
-    </row>
-    <row r="4" spans="1:18" ht="12.75" customHeight="1" ns2:dyDescent="0.2">
+      <c r="M3" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+    </row>
+    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
-      <c r="M4" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="29"/>
-      <c r="R4" s="29"/>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" ns2:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="M4" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="27"/>
+    </row>
+    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" ns2:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-    </row>
-    <row r="8" spans="1:18" s="3" customFormat="1" ht="30" customHeight="1" ns2:dyDescent="0.2">
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+    </row>
+    <row r="8" spans="1:18" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="23" t="s">
         <v>0</v>
       </c>
@@ -886,13 +886,13 @@
         <v>28</v>
       </c>
       <c r="Q8" s="23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="R8" s="23" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="3" customFormat="1" ht="46.5" customHeight="1" ns2:dyDescent="0.2">
+    <row r="9" spans="1:18" s="3" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
@@ -930,7 +930,7 @@
       <c r="Q9" s="23"/>
       <c r="R9" s="23"/>
     </row>
-    <row r="10" spans="1:18" s="5" customFormat="1" ns2:dyDescent="0.2">
+    <row r="10" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="17" t="s">
         <v>4</v>
       </c>
@@ -986,10 +986,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="19.5" customHeight="1" ns2:dyDescent="0.2">
+    <row r="11" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6"/>
       <c r="B11" s="14" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -1008,12 +1008,12 @@
       <c r="Q11" s="15"/>
       <c r="R11" s="15"/>
     </row>
-    <row r="12" spans="1:18" s="8" customFormat="1" ht="63" customHeight="1" ns2:dyDescent="0.2">
+    <row r="12" spans="1:18" s="8" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>32</v>
@@ -1040,10 +1040,10 @@
         <v>39</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="M12" s="19" t="s">
         <v>40</v>
@@ -1052,7 +1052,7 @@
         <v>41</v>
       </c>
       <c r="O12" s="19" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="P12" s="19" t="s">
         <v>42</v>
@@ -1061,94 +1061,106 @@
         <v>43</v>
       </c>
       <c r="R12" s="19" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
       <c r="G14" s="11"/>
-      <c r="K14" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="L14" s="22"/>
-      <c r="M14" s="22"/>
-      <c r="N14" s="22"/>
-      <c r="O14" s="22"/>
-      <c r="P14" s="22"/>
-    </row>
-    <row r="15" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="K14" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="L14" s="29"/>
+      <c r="M14" s="29"/>
+      <c r="N14" s="29"/>
+      <c r="O14" s="29"/>
+      <c r="P14" s="29"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="9"/>
-      <c r="K15" s="21" t="s">
+      <c r="K15" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="L15" s="21"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="21"/>
-      <c r="P15" s="21"/>
-    </row>
-    <row r="16" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
+      <c r="L15" s="28"/>
+      <c r="M15" s="28"/>
+      <c r="N15" s="28"/>
+      <c r="O15" s="28"/>
+      <c r="P15" s="28"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="9"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="21"/>
-      <c r="P16" s="21"/>
-    </row>
-    <row r="17" spans="1:16" ns2:dyDescent="0.2">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
+      <c r="M16" s="28"/>
+      <c r="N16" s="28"/>
+      <c r="O16" s="28"/>
+      <c r="P16" s="28"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
       <c r="G17" s="9"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="21"/>
-      <c r="P17" s="21"/>
-    </row>
-    <row r="18" spans="1:16" ns2:dyDescent="0.2">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
+      <c r="K17" s="28"/>
+      <c r="L17" s="28"/>
+      <c r="M17" s="28"/>
+      <c r="N17" s="28"/>
+      <c r="O17" s="28"/>
+      <c r="P17" s="28"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
       <c r="G18" s="9"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
-      <c r="P18" s="21"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
+      <c r="M18" s="28"/>
+      <c r="N18" s="28"/>
+      <c r="O18" s="28"/>
+      <c r="P18" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="K15:P18"/>
+    <mergeCell ref="A15:F18"/>
+    <mergeCell ref="K14:P14"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="M8:M9"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A8:A9"/>
@@ -1163,21 +1175,9 @@
     <mergeCell ref="M2:R2"/>
     <mergeCell ref="Q8:Q9"/>
     <mergeCell ref="R8:R9"/>
-    <mergeCell ref="K15:P18"/>
-    <mergeCell ref="A15:F18"/>
-    <mergeCell ref="K14:P14"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="M8:M9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="3" fitToWidth="1" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="3" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>